<commit_message>
Ajuste na data do Resumo Semanal, limpeza do código de Cartão de Trabalho e atualizações gerais
</commit_message>
<xml_diff>
--- a/Planejamento Previsto Geral.xlsx
+++ b/Planejamento Previsto Geral.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E121F774-3B22-4AE4-8C9B-5894E1D622A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08A0151-7658-494E-A9A9-04D47BBF4E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="6" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="37">
   <si>
     <t>ATIVIDADE</t>
   </si>
@@ -121,6 +121,24 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>Reaterro compactado (m²)</t>
+  </si>
+  <si>
+    <t>Escavação (m)</t>
+  </si>
+  <si>
+    <t>Remoção de pavimento asfáltico (m)</t>
+  </si>
+  <si>
+    <t>Reposição de pavimento asfáltico (m)</t>
+  </si>
+  <si>
+    <t>Remoção de pavimento granitico (m)</t>
   </si>
 </sst>
 </file>
@@ -712,58 +730,79 @@
     <xf numFmtId="165" fontId="4" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -772,64 +811,43 @@
     <xf numFmtId="1" fontId="1" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1166,7 +1184,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:BN59"/>
+  <dimension ref="B1:BN61"/>
   <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="1.6640625" customWidth="1"/>
@@ -1200,104 +1218,104 @@
   <sheetData>
     <row r="1" spans="2:66" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:66" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="50" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="48" t="s">
+      <c r="B2" s="74" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="48" t="s">
+      <c r="E2" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="48" t="s">
+      <c r="F2" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="48" t="s">
+      <c r="G2" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="48" t="s">
+      <c r="H2" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="47" t="s">
+      <c r="I2" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="48" t="s">
+      <c r="J2" s="76"/>
+      <c r="K2" s="76"/>
+      <c r="L2" s="76"/>
+      <c r="M2" s="76"/>
+      <c r="N2" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="48"/>
-      <c r="P2" s="48"/>
-      <c r="Q2" s="48"/>
-      <c r="R2" s="48"/>
-      <c r="S2" s="48" t="s">
+      <c r="O2" s="76"/>
+      <c r="P2" s="76"/>
+      <c r="Q2" s="76"/>
+      <c r="R2" s="76"/>
+      <c r="S2" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="T2" s="48"/>
-      <c r="U2" s="48"/>
-      <c r="V2" s="48"/>
-      <c r="W2" s="48"/>
-      <c r="X2" s="48"/>
-      <c r="Y2" s="48" t="s">
+      <c r="T2" s="76"/>
+      <c r="U2" s="76"/>
+      <c r="V2" s="76"/>
+      <c r="W2" s="76"/>
+      <c r="X2" s="76"/>
+      <c r="Y2" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="Z2" s="48"/>
-      <c r="AA2" s="48"/>
-      <c r="AB2" s="48"/>
-      <c r="AC2" s="48"/>
-      <c r="AD2" s="48"/>
-      <c r="AE2" s="48" t="s">
+      <c r="Z2" s="76"/>
+      <c r="AA2" s="76"/>
+      <c r="AB2" s="76"/>
+      <c r="AC2" s="76"/>
+      <c r="AD2" s="76"/>
+      <c r="AE2" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="AF2" s="48"/>
-      <c r="AG2" s="48"/>
-      <c r="AH2" s="48"/>
-      <c r="AI2" s="48"/>
-      <c r="AJ2" s="48" t="s">
+      <c r="AF2" s="76"/>
+      <c r="AG2" s="76"/>
+      <c r="AH2" s="76"/>
+      <c r="AI2" s="76"/>
+      <c r="AJ2" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="AK2" s="48"/>
-      <c r="AL2" s="48"/>
-      <c r="AM2" s="48"/>
-      <c r="AN2" s="48"/>
-      <c r="AO2" s="48"/>
-      <c r="AP2" s="48" t="s">
+      <c r="AK2" s="76"/>
+      <c r="AL2" s="76"/>
+      <c r="AM2" s="76"/>
+      <c r="AN2" s="76"/>
+      <c r="AO2" s="76"/>
+      <c r="AP2" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="AQ2" s="48"/>
-      <c r="AR2" s="48"/>
-      <c r="AS2" s="48"/>
-      <c r="AT2" s="48"/>
-      <c r="AU2" s="48"/>
-      <c r="AV2" s="48" t="s">
+      <c r="AQ2" s="76"/>
+      <c r="AR2" s="76"/>
+      <c r="AS2" s="76"/>
+      <c r="AT2" s="76"/>
+      <c r="AU2" s="76"/>
+      <c r="AV2" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="AW2" s="48"/>
-      <c r="AX2" s="48"/>
-      <c r="AY2" s="48"/>
-      <c r="AZ2" s="48"/>
-      <c r="BA2" s="48"/>
-      <c r="BB2" s="48" t="s">
+      <c r="AW2" s="76"/>
+      <c r="AX2" s="76"/>
+      <c r="AY2" s="76"/>
+      <c r="AZ2" s="76"/>
+      <c r="BA2" s="76"/>
+      <c r="BB2" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="BC2" s="48"/>
-      <c r="BD2" s="48"/>
-      <c r="BE2" s="48"/>
-      <c r="BF2" s="49"/>
+      <c r="BC2" s="76"/>
+      <c r="BD2" s="76"/>
+      <c r="BE2" s="76"/>
+      <c r="BF2" s="86"/>
     </row>
     <row r="3" spans="2:66" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="51"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
+      <c r="B3" s="75"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
       <c r="I3" s="4">
         <v>46083</v>
       </c>
@@ -1453,17 +1471,17 @@
       <c r="B4" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="57">
+      <c r="C4" s="80">
         <v>1</v>
       </c>
-      <c r="D4" s="60">
+      <c r="D4" s="83">
         <f>SUM(K4:AC4)</f>
         <v>800</v>
       </c>
-      <c r="E4" s="62">
+      <c r="E4" s="60">
         <v>46083</v>
       </c>
-      <c r="F4" s="62">
+      <c r="F4" s="60">
         <v>46122</v>
       </c>
       <c r="G4" s="7" t="s">
@@ -1579,17 +1597,17 @@
       <c r="BN4" s="14"/>
     </row>
     <row r="5" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B5" s="56"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="64"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="84"/>
       <c r="G5" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H5" s="15">
         <f t="shared" ref="H5:H59" si="0">SUM(I5:BF5)</f>
-        <v>829</v>
+        <v>869</v>
       </c>
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
@@ -1657,14 +1675,20 @@
       <c r="AJ5" s="17">
         <v>30</v>
       </c>
-      <c r="AK5" s="17"/>
-      <c r="AL5" s="16"/>
+      <c r="AK5" s="17">
+        <v>40</v>
+      </c>
+      <c r="AL5" s="16">
+        <v>256</v>
+      </c>
       <c r="AM5" s="17"/>
       <c r="AN5" s="17"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="17"/>
       <c r="AQ5" s="17"/>
-      <c r="AR5" s="17"/>
+      <c r="AR5" s="17">
+        <v>-256</v>
+      </c>
       <c r="AS5" s="17"/>
       <c r="AT5" s="17"/>
       <c r="AU5" s="17"/>
@@ -1689,18 +1713,18 @@
       <c r="BN5" s="14"/>
     </row>
     <row r="6" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="58"/>
-      <c r="D6" s="61">
+      <c r="C6" s="81"/>
+      <c r="D6" s="66">
         <f>SUM(Y6:AC6)</f>
         <v>325</v>
       </c>
-      <c r="E6" s="63">
+      <c r="E6" s="49">
         <v>46083</v>
       </c>
-      <c r="F6" s="63">
+      <c r="F6" s="49">
         <v>46122</v>
       </c>
       <c r="G6" s="19" t="s">
@@ -1806,17 +1830,17 @@
       <c r="BN6" s="14"/>
     </row>
     <row r="7" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B7" s="56"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="61"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
       <c r="G7" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H7" s="15">
         <f t="shared" si="0"/>
-        <v>829</v>
+        <v>869</v>
       </c>
       <c r="I7" s="16"/>
       <c r="J7" s="16"/>
@@ -1870,14 +1894,20 @@
       <c r="AJ7" s="17">
         <v>30</v>
       </c>
-      <c r="AK7" s="17"/>
-      <c r="AL7" s="16"/>
+      <c r="AK7" s="17">
+        <v>40</v>
+      </c>
+      <c r="AL7" s="16">
+        <v>256</v>
+      </c>
       <c r="AM7" s="17"/>
       <c r="AN7" s="17"/>
       <c r="AO7" s="17"/>
       <c r="AP7" s="17"/>
       <c r="AQ7" s="17"/>
-      <c r="AR7" s="17"/>
+      <c r="AR7" s="17">
+        <v>-256</v>
+      </c>
       <c r="AS7" s="17"/>
       <c r="AT7" s="17"/>
       <c r="AU7" s="17"/>
@@ -1902,18 +1932,18 @@
       <c r="BN7" s="14"/>
     </row>
     <row r="8" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="58"/>
-      <c r="D8" s="61">
+      <c r="C8" s="81"/>
+      <c r="D8" s="66">
         <f>SUM(N8:AD8)</f>
         <v>422.00000000000011</v>
       </c>
-      <c r="E8" s="63">
+      <c r="E8" s="49">
         <v>46083</v>
       </c>
-      <c r="F8" s="63">
+      <c r="F8" s="49">
         <v>46122</v>
       </c>
       <c r="G8" s="15" t="s">
@@ -2027,17 +2057,17 @@
       <c r="BN8" s="14"/>
     </row>
     <row r="9" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B9" s="56"/>
-      <c r="C9" s="58"/>
-      <c r="D9" s="61"/>
-      <c r="E9" s="63"/>
-      <c r="F9" s="63"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="81"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
       <c r="G9" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H9" s="15">
         <f t="shared" si="0"/>
-        <v>441.9</v>
+        <v>473.4</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
@@ -2098,7 +2128,9 @@
       <c r="AI9" s="16"/>
       <c r="AJ9" s="17"/>
       <c r="AK9" s="17"/>
-      <c r="AL9" s="16"/>
+      <c r="AL9" s="16">
+        <v>31.5</v>
+      </c>
       <c r="AM9" s="17"/>
       <c r="AN9" s="17"/>
       <c r="AO9" s="17"/>
@@ -2129,18 +2161,18 @@
       <c r="BN9" s="14"/>
     </row>
     <row r="10" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B10" s="56" t="s">
+      <c r="B10" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="58"/>
-      <c r="D10" s="61">
+      <c r="C10" s="81"/>
+      <c r="D10" s="66">
         <f>SUM(O10:AK10)</f>
         <v>63.3</v>
       </c>
-      <c r="E10" s="63">
+      <c r="E10" s="49">
         <v>46084</v>
       </c>
-      <c r="F10" s="63">
+      <c r="F10" s="49">
         <v>46125</v>
       </c>
       <c r="G10" s="15" t="s">
@@ -2264,17 +2296,17 @@
       <c r="BN10" s="14"/>
     </row>
     <row r="11" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B11" s="56"/>
-      <c r="C11" s="58"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="81"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
       <c r="G11" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H11" s="15">
         <f t="shared" si="0"/>
-        <v>92.759999999999991</v>
+        <v>94.259999999999991</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="16"/>
@@ -2341,7 +2373,9 @@
         <v>1.5</v>
       </c>
       <c r="AK11" s="17"/>
-      <c r="AL11" s="16"/>
+      <c r="AL11" s="16">
+        <v>1.5</v>
+      </c>
       <c r="AM11" s="17"/>
       <c r="AN11" s="17"/>
       <c r="AO11" s="17"/>
@@ -2372,18 +2406,18 @@
       <c r="BN11" s="14"/>
     </row>
     <row r="12" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B12" s="65" t="s">
+      <c r="B12" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="58"/>
-      <c r="D12" s="66">
+      <c r="C12" s="81"/>
+      <c r="D12" s="73">
         <f>SUM(N12:AN12)</f>
         <v>400</v>
       </c>
-      <c r="E12" s="63">
+      <c r="E12" s="49">
         <v>46085</v>
       </c>
-      <c r="F12" s="63">
+      <c r="F12" s="49">
         <v>46126</v>
       </c>
       <c r="G12" s="15" t="s">
@@ -2510,17 +2544,17 @@
       <c r="BN12" s="14"/>
     </row>
     <row r="13" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B13" s="65"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="81"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
       <c r="G13" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H13" s="15">
         <f t="shared" si="0"/>
-        <v>354</v>
+        <v>400</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="16"/>
@@ -2587,12 +2621,18 @@
       <c r="AK13" s="17">
         <v>36</v>
       </c>
-      <c r="AL13" s="16"/>
-      <c r="AM13" s="17"/>
+      <c r="AL13" s="16">
+        <v>18</v>
+      </c>
+      <c r="AM13" s="17">
+        <v>30</v>
+      </c>
       <c r="AN13" s="17"/>
       <c r="AO13" s="17"/>
       <c r="AP13" s="17"/>
-      <c r="AQ13" s="17"/>
+      <c r="AQ13" s="17">
+        <v>-2</v>
+      </c>
       <c r="AR13" s="17"/>
       <c r="AS13" s="17"/>
       <c r="AT13" s="17"/>
@@ -2618,18 +2658,18 @@
       <c r="BN13" s="14"/>
     </row>
     <row r="14" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B14" s="56" t="s">
+      <c r="B14" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="58"/>
-      <c r="D14" s="61">
+      <c r="C14" s="81"/>
+      <c r="D14" s="66">
         <f>SUM(R14:AM14)</f>
         <v>5</v>
       </c>
-      <c r="E14" s="63">
+      <c r="E14" s="49">
         <v>46090</v>
       </c>
-      <c r="F14" s="63">
+      <c r="F14" s="49">
         <v>46126</v>
       </c>
       <c r="G14" s="15" t="s">
@@ -2719,17 +2759,17 @@
       <c r="BN14" s="14"/>
     </row>
     <row r="15" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B15" s="56"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="61"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
       <c r="G15" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H15" s="15">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I15" s="16"/>
       <c r="J15" s="16"/>
@@ -2768,7 +2808,9 @@
       <c r="AI15" s="16"/>
       <c r="AJ15" s="17"/>
       <c r="AK15" s="17"/>
-      <c r="AL15" s="16"/>
+      <c r="AL15" s="16">
+        <v>1</v>
+      </c>
       <c r="AM15" s="17"/>
       <c r="AN15" s="17"/>
       <c r="AO15" s="17"/>
@@ -2799,18 +2841,18 @@
       <c r="BN15" s="14"/>
     </row>
     <row r="16" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B16" s="56" t="s">
+      <c r="B16" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="58"/>
-      <c r="D16" s="61">
+      <c r="C16" s="81"/>
+      <c r="D16" s="66">
         <f>SUM(N16:AN16)</f>
         <v>372</v>
       </c>
-      <c r="E16" s="63">
+      <c r="E16" s="49">
         <v>46085</v>
       </c>
-      <c r="F16" s="63">
+      <c r="F16" s="49">
         <v>46127</v>
       </c>
       <c r="G16" s="15" t="s">
@@ -2942,17 +2984,17 @@
       <c r="BN16" s="14"/>
     </row>
     <row r="17" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B17" s="56"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="81"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
       <c r="G17" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H17" s="15">
         <f t="shared" si="0"/>
-        <v>347.27</v>
+        <v>425.32</v>
       </c>
       <c r="I17" s="16"/>
       <c r="J17" s="16"/>
@@ -3013,9 +3055,13 @@
       <c r="AI17" s="16"/>
       <c r="AJ17" s="17"/>
       <c r="AK17" s="17"/>
-      <c r="AL17" s="16"/>
+      <c r="AL17" s="16">
+        <v>37.6</v>
+      </c>
       <c r="AM17" s="17"/>
-      <c r="AN17" s="17"/>
+      <c r="AN17" s="17">
+        <v>40.450000000000003</v>
+      </c>
       <c r="AO17" s="17"/>
       <c r="AP17" s="17"/>
       <c r="AQ17" s="17"/>
@@ -3044,18 +3090,18 @@
       <c r="BN17" s="14"/>
     </row>
     <row r="18" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="58"/>
-      <c r="D18" s="61">
+      <c r="C18" s="81"/>
+      <c r="D18" s="66">
         <f>SUM(R18:AO18)</f>
         <v>285</v>
       </c>
-      <c r="E18" s="63">
+      <c r="E18" s="49">
         <v>46090</v>
       </c>
-      <c r="F18" s="63">
+      <c r="F18" s="49">
         <v>46129</v>
       </c>
       <c r="G18" s="15" t="s">
@@ -3153,17 +3199,17 @@
       <c r="BN18" s="14"/>
     </row>
     <row r="19" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B19" s="56"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="61"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="81"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49"/>
       <c r="G19" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H19" s="15">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>341.4</v>
       </c>
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
@@ -3200,9 +3246,15 @@
         <v>50</v>
       </c>
       <c r="AK19" s="17"/>
-      <c r="AL19" s="16"/>
-      <c r="AM19" s="17"/>
-      <c r="AN19" s="17"/>
+      <c r="AL19" s="16">
+        <v>132.5</v>
+      </c>
+      <c r="AM19" s="17">
+        <v>117.5</v>
+      </c>
+      <c r="AN19" s="17">
+        <v>41.4</v>
+      </c>
       <c r="AO19" s="17"/>
       <c r="AP19" s="17"/>
       <c r="AQ19" s="17"/>
@@ -3231,18 +3283,18 @@
       <c r="BN19" s="14"/>
     </row>
     <row r="20" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B20" s="56" t="s">
+      <c r="B20" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="58"/>
-      <c r="D20" s="61">
+      <c r="C20" s="81"/>
+      <c r="D20" s="66">
         <f>SUM(Z20:AS20)</f>
         <v>800</v>
       </c>
-      <c r="E20" s="63">
+      <c r="E20" s="49">
         <v>46097</v>
       </c>
-      <c r="F20" s="63">
+      <c r="F20" s="49">
         <v>46134</v>
       </c>
       <c r="G20" s="15" t="s">
@@ -3326,17 +3378,17 @@
       <c r="BN20" s="14"/>
     </row>
     <row r="21" spans="2:66" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="67"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="68"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
+      <c r="B21" s="50"/>
+      <c r="C21" s="82"/>
+      <c r="D21" s="67"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
       <c r="G21" s="31" t="s">
         <v>20</v>
       </c>
       <c r="H21" s="31">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>341.4</v>
       </c>
       <c r="I21" s="32"/>
       <c r="J21" s="32"/>
@@ -3373,9 +3425,15 @@
         <v>50</v>
       </c>
       <c r="AK21" s="33"/>
-      <c r="AL21" s="32"/>
-      <c r="AM21" s="33"/>
-      <c r="AN21" s="33"/>
+      <c r="AL21" s="32">
+        <v>132.5</v>
+      </c>
+      <c r="AM21" s="33">
+        <v>117.5</v>
+      </c>
+      <c r="AN21" s="33">
+        <v>41.4</v>
+      </c>
       <c r="AO21" s="33"/>
       <c r="AP21" s="33"/>
       <c r="AQ21" s="33"/>
@@ -3399,17 +3457,17 @@
       <c r="B22" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="70">
+      <c r="C22" s="68">
         <v>2</v>
       </c>
-      <c r="D22" s="73">
+      <c r="D22" s="71">
         <f>AA22</f>
         <v>5</v>
       </c>
-      <c r="E22" s="62">
+      <c r="E22" s="60">
         <v>46097</v>
       </c>
-      <c r="F22" s="62">
+      <c r="F22" s="60">
         <v>46134</v>
       </c>
       <c r="G22" s="35" t="s">
@@ -3483,11 +3541,11 @@
       </c>
     </row>
     <row r="23" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B23" s="56"/>
-      <c r="C23" s="71"/>
-      <c r="D23" s="74"/>
-      <c r="E23" s="63"/>
-      <c r="F23" s="63"/>
+      <c r="B23" s="47"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
       <c r="G23" s="15" t="s">
         <v>20</v>
       </c>
@@ -3549,18 +3607,18 @@
       <c r="BF23" s="18"/>
     </row>
     <row r="24" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B24" s="56" t="s">
+      <c r="B24" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="71"/>
-      <c r="D24" s="74">
+      <c r="C24" s="69"/>
+      <c r="D24" s="63">
         <f>SUM(AB24:AK24)</f>
         <v>204</v>
       </c>
-      <c r="E24" s="63">
+      <c r="E24" s="49">
         <v>46097</v>
       </c>
-      <c r="F24" s="63">
+      <c r="F24" s="49">
         <v>46134</v>
       </c>
       <c r="G24" s="15" t="s">
@@ -3652,17 +3710,17 @@
       </c>
     </row>
     <row r="25" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B25" s="56"/>
-      <c r="C25" s="71"/>
-      <c r="D25" s="74"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
+      <c r="B25" s="47"/>
+      <c r="C25" s="69"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
       <c r="G25" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H25" s="15">
         <f t="shared" si="0"/>
-        <v>149.5</v>
+        <v>343.5</v>
       </c>
       <c r="I25" s="16"/>
       <c r="J25" s="16"/>
@@ -3699,7 +3757,9 @@
       <c r="AK25" s="17"/>
       <c r="AL25" s="16"/>
       <c r="AM25" s="17"/>
-      <c r="AN25" s="17"/>
+      <c r="AN25" s="17">
+        <v>194</v>
+      </c>
       <c r="AO25" s="17"/>
       <c r="AP25" s="17"/>
       <c r="AQ25" s="17"/>
@@ -3720,18 +3780,18 @@
       <c r="BF25" s="18"/>
     </row>
     <row r="26" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B26" s="56" t="s">
+      <c r="B26" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="71"/>
-      <c r="D26" s="74">
+      <c r="C26" s="69"/>
+      <c r="D26" s="63">
         <f>SUM(AB26:AK26)</f>
         <v>204</v>
       </c>
-      <c r="E26" s="63">
+      <c r="E26" s="49">
         <v>46097</v>
       </c>
-      <c r="F26" s="63">
+      <c r="F26" s="49">
         <v>46134</v>
       </c>
       <c r="G26" s="15" t="s">
@@ -3823,17 +3883,17 @@
       </c>
     </row>
     <row r="27" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B27" s="56"/>
-      <c r="C27" s="71"/>
-      <c r="D27" s="74"/>
-      <c r="E27" s="63"/>
-      <c r="F27" s="63"/>
+      <c r="B27" s="47"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="63"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
       <c r="G27" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H27" s="15">
         <f t="shared" si="0"/>
-        <v>149.5</v>
+        <v>343.5</v>
       </c>
       <c r="I27" s="16"/>
       <c r="J27" s="16"/>
@@ -3870,7 +3930,9 @@
       <c r="AK27" s="17"/>
       <c r="AL27" s="16"/>
       <c r="AM27" s="17"/>
-      <c r="AN27" s="17"/>
+      <c r="AN27" s="17">
+        <v>194</v>
+      </c>
       <c r="AO27" s="17"/>
       <c r="AP27" s="17"/>
       <c r="AQ27" s="17"/>
@@ -3891,18 +3953,18 @@
       <c r="BF27" s="18"/>
     </row>
     <row r="28" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B28" s="56" t="s">
+      <c r="B28" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="C28" s="71"/>
-      <c r="D28" s="74">
+      <c r="C28" s="69"/>
+      <c r="D28" s="63">
         <f>SUM(AC28:AH28,AK28:AP28)</f>
         <v>155.6</v>
       </c>
-      <c r="E28" s="63">
+      <c r="E28" s="49">
         <v>46097</v>
       </c>
-      <c r="F28" s="63">
+      <c r="F28" s="49">
         <v>46134</v>
       </c>
       <c r="G28" s="15" t="s">
@@ -4006,17 +4068,17 @@
       </c>
     </row>
     <row r="29" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B29" s="56"/>
-      <c r="C29" s="71"/>
-      <c r="D29" s="74"/>
-      <c r="E29" s="63"/>
-      <c r="F29" s="63"/>
+      <c r="B29" s="47"/>
+      <c r="C29" s="69"/>
+      <c r="D29" s="63"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
       <c r="G29" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H29" s="15">
         <f t="shared" si="0"/>
-        <v>35.28</v>
+        <v>189.68</v>
       </c>
       <c r="I29" s="16"/>
       <c r="J29" s="16"/>
@@ -4048,12 +4110,22 @@
       <c r="AJ29" s="17">
         <v>35.28</v>
       </c>
-      <c r="AK29" s="17"/>
+      <c r="AK29" s="17">
+        <v>16</v>
+      </c>
       <c r="AL29" s="16"/>
-      <c r="AM29" s="17"/>
-      <c r="AN29" s="17"/>
-      <c r="AO29" s="17"/>
-      <c r="AP29" s="17"/>
+      <c r="AM29" s="17">
+        <v>25</v>
+      </c>
+      <c r="AN29" s="17">
+        <v>45.36</v>
+      </c>
+      <c r="AO29" s="17">
+        <v>30.24</v>
+      </c>
+      <c r="AP29" s="17">
+        <v>37.799999999999997</v>
+      </c>
       <c r="AQ29" s="17"/>
       <c r="AR29" s="17"/>
       <c r="AS29" s="17"/>
@@ -4072,18 +4144,18 @@
       <c r="BF29" s="18"/>
     </row>
     <row r="30" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B30" s="56" t="s">
+      <c r="B30" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="71"/>
-      <c r="D30" s="74">
+      <c r="C30" s="69"/>
+      <c r="D30" s="63">
         <f>SUM(AD30:AH30,AJ30:BE30)</f>
         <v>19.779999999999998</v>
       </c>
-      <c r="E30" s="63">
+      <c r="E30" s="49">
         <v>46097</v>
       </c>
-      <c r="F30" s="63">
+      <c r="F30" s="49">
         <v>46134</v>
       </c>
       <c r="G30" s="15" t="s">
@@ -4169,17 +4241,17 @@
       </c>
     </row>
     <row r="31" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B31" s="56"/>
-      <c r="C31" s="71"/>
-      <c r="D31" s="74"/>
-      <c r="E31" s="63"/>
-      <c r="F31" s="63"/>
+      <c r="B31" s="47"/>
+      <c r="C31" s="69"/>
+      <c r="D31" s="63"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="49"/>
       <c r="G31" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H31" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>8.64</v>
       </c>
       <c r="I31" s="16"/>
       <c r="J31" s="16"/>
@@ -4213,7 +4285,9 @@
       <c r="AL31" s="16"/>
       <c r="AM31" s="17"/>
       <c r="AN31" s="17"/>
-      <c r="AO31" s="17"/>
+      <c r="AO31" s="17">
+        <v>8.64</v>
+      </c>
       <c r="AP31" s="17"/>
       <c r="AQ31" s="17"/>
       <c r="AR31" s="17"/>
@@ -4233,18 +4307,18 @@
       <c r="BF31" s="18"/>
     </row>
     <row r="32" spans="2:66" x14ac:dyDescent="0.3">
-      <c r="B32" s="75" t="s">
+      <c r="B32" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="C32" s="71"/>
-      <c r="D32" s="76">
+      <c r="C32" s="69"/>
+      <c r="D32" s="65">
         <f>SUM(AE32:AH32,AJ32:AW32)</f>
         <v>238</v>
       </c>
-      <c r="E32" s="63">
+      <c r="E32" s="49">
         <v>46097</v>
       </c>
-      <c r="F32" s="63">
+      <c r="F32" s="49">
         <v>46134</v>
       </c>
       <c r="G32" s="15" t="s">
@@ -4346,17 +4420,17 @@
       </c>
     </row>
     <row r="33" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B33" s="75"/>
-      <c r="C33" s="71"/>
-      <c r="D33" s="76"/>
-      <c r="E33" s="63"/>
-      <c r="F33" s="63"/>
+      <c r="B33" s="64"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="65"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
       <c r="G33" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H33" s="15">
         <f t="shared" si="0"/>
-        <v>36</v>
+        <v>110</v>
       </c>
       <c r="I33" s="16"/>
       <c r="J33" s="16"/>
@@ -4389,11 +4463,19 @@
       <c r="AK33" s="17">
         <v>36</v>
       </c>
-      <c r="AL33" s="16"/>
-      <c r="AM33" s="17"/>
+      <c r="AL33" s="16">
+        <v>12</v>
+      </c>
+      <c r="AM33" s="17">
+        <v>20</v>
+      </c>
       <c r="AN33" s="17"/>
-      <c r="AO33" s="17"/>
-      <c r="AP33" s="17"/>
+      <c r="AO33" s="17">
+        <v>12</v>
+      </c>
+      <c r="AP33" s="17">
+        <v>30</v>
+      </c>
       <c r="AQ33" s="17"/>
       <c r="AR33" s="17"/>
       <c r="AS33" s="17"/>
@@ -4412,18 +4494,18 @@
       <c r="BF33" s="18"/>
     </row>
     <row r="34" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B34" s="56" t="s">
+      <c r="B34" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="C34" s="71"/>
-      <c r="D34" s="77">
+      <c r="C34" s="69"/>
+      <c r="D34" s="53">
         <f>SUM(AJ34:AW34)</f>
         <v>3</v>
       </c>
-      <c r="E34" s="63">
+      <c r="E34" s="49">
         <v>46097</v>
       </c>
-      <c r="F34" s="63">
+      <c r="F34" s="49">
         <v>46134</v>
       </c>
       <c r="G34" s="15" t="s">
@@ -4501,11 +4583,11 @@
       </c>
     </row>
     <row r="35" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B35" s="56"/>
-      <c r="C35" s="71"/>
-      <c r="D35" s="77"/>
-      <c r="E35" s="63"/>
-      <c r="F35" s="63"/>
+      <c r="B35" s="47"/>
+      <c r="C35" s="69"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="49"/>
       <c r="G35" s="15" t="s">
         <v>20</v>
       </c>
@@ -4565,18 +4647,18 @@
       <c r="BF35" s="18"/>
     </row>
     <row r="36" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B36" s="56" t="s">
+      <c r="B36" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C36" s="71"/>
-      <c r="D36" s="77">
+      <c r="C36" s="69"/>
+      <c r="D36" s="53">
         <f>SUM(AE36:AH36,AJ36:AU36)</f>
         <v>192</v>
       </c>
-      <c r="E36" s="63">
+      <c r="E36" s="49">
         <v>46097</v>
       </c>
-      <c r="F36" s="63">
+      <c r="F36" s="49">
         <v>46134</v>
       </c>
       <c r="G36" s="15" t="s">
@@ -4686,17 +4768,17 @@
       </c>
     </row>
     <row r="37" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B37" s="56"/>
-      <c r="C37" s="71"/>
-      <c r="D37" s="77"/>
-      <c r="E37" s="63"/>
-      <c r="F37" s="63"/>
+      <c r="B37" s="47"/>
+      <c r="C37" s="69"/>
+      <c r="D37" s="53"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
       <c r="G37" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H37" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>79.97999999999999</v>
       </c>
       <c r="I37" s="16"/>
       <c r="J37" s="16"/>
@@ -4729,9 +4811,15 @@
       <c r="AK37" s="17"/>
       <c r="AL37" s="16"/>
       <c r="AM37" s="17"/>
-      <c r="AN37" s="17"/>
-      <c r="AO37" s="17"/>
-      <c r="AP37" s="17"/>
+      <c r="AN37" s="17">
+        <v>46.5</v>
+      </c>
+      <c r="AO37" s="17">
+        <v>11.16</v>
+      </c>
+      <c r="AP37" s="17">
+        <v>22.32</v>
+      </c>
       <c r="AQ37" s="17"/>
       <c r="AR37" s="17"/>
       <c r="AS37" s="17"/>
@@ -4750,18 +4838,18 @@
       <c r="BF37" s="18"/>
     </row>
     <row r="38" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B38" s="56" t="s">
+      <c r="B38" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="71"/>
-      <c r="D38" s="77">
+      <c r="C38" s="69"/>
+      <c r="D38" s="53">
         <f>SUM(AJ38:AU38)</f>
         <v>280</v>
       </c>
-      <c r="E38" s="63">
+      <c r="E38" s="49">
         <v>46097</v>
       </c>
-      <c r="F38" s="63">
+      <c r="F38" s="49">
         <v>46134</v>
       </c>
       <c r="G38" s="15" t="s">
@@ -4857,11 +4945,11 @@
       </c>
     </row>
     <row r="39" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B39" s="56"/>
-      <c r="C39" s="71"/>
-      <c r="D39" s="77"/>
-      <c r="E39" s="63"/>
-      <c r="F39" s="63"/>
+      <c r="B39" s="47"/>
+      <c r="C39" s="69"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
       <c r="G39" s="15" t="s">
         <v>20</v>
       </c>
@@ -4921,18 +5009,18 @@
       <c r="BF39" s="18"/>
     </row>
     <row r="40" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B40" s="56" t="s">
+      <c r="B40" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="C40" s="71"/>
-      <c r="D40" s="77">
+      <c r="C40" s="69"/>
+      <c r="D40" s="53">
         <f>SUM(AU40:AZ40)</f>
-        <v>160</v>
-      </c>
-      <c r="E40" s="63">
+        <v>250</v>
+      </c>
+      <c r="E40" s="49">
         <v>46097</v>
       </c>
-      <c r="F40" s="63">
+      <c r="F40" s="49">
         <v>46134</v>
       </c>
       <c r="G40" s="15" t="s">
@@ -4996,12 +5084,12 @@
       <c r="AX40" s="26"/>
       <c r="AY40" s="26"/>
       <c r="AZ40" s="40">
-        <v>160</v>
+        <v>250</v>
       </c>
       <c r="BA40" s="26"/>
       <c r="BB40" s="26"/>
       <c r="BC40" s="26">
-        <v>316</v>
+        <v>226</v>
       </c>
       <c r="BD40" s="26"/>
       <c r="BE40" s="26"/>
@@ -5010,11 +5098,11 @@
       </c>
     </row>
     <row r="41" spans="2:58" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="67"/>
-      <c r="C41" s="72"/>
-      <c r="D41" s="78"/>
-      <c r="E41" s="69"/>
-      <c r="F41" s="69"/>
+      <c r="B41" s="50"/>
+      <c r="C41" s="70"/>
+      <c r="D41" s="54"/>
+      <c r="E41" s="52"/>
+      <c r="F41" s="52"/>
       <c r="G41" s="31" t="s">
         <v>20</v>
       </c>
@@ -5075,19 +5163,19 @@
     </row>
     <row r="42" spans="2:58" x14ac:dyDescent="0.3">
       <c r="B42" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42" s="79">
+        <v>36</v>
+      </c>
+      <c r="C42" s="56">
         <v>3</v>
       </c>
-      <c r="D42" s="82">
+      <c r="D42" s="59">
         <f>SUM(AJ42:AK42)</f>
         <v>0</v>
       </c>
-      <c r="E42" s="62">
+      <c r="E42" s="60">
         <v>46097</v>
       </c>
-      <c r="F42" s="62">
+      <c r="F42" s="60">
         <v>46134</v>
       </c>
       <c r="G42" s="35" t="s">
@@ -5095,7 +5183,7 @@
       </c>
       <c r="H42" s="35">
         <f t="shared" si="0"/>
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="I42" s="36"/>
       <c r="J42" s="37"/>
@@ -5138,12 +5226,8 @@
       <c r="AM42" s="37"/>
       <c r="AN42" s="37"/>
       <c r="AO42" s="37"/>
-      <c r="AP42" s="37">
-        <v>63</v>
-      </c>
-      <c r="AQ42" s="37">
-        <v>63</v>
-      </c>
+      <c r="AP42" s="37"/>
+      <c r="AQ42" s="37"/>
       <c r="AR42" s="37"/>
       <c r="AS42" s="37"/>
       <c r="AT42" s="37"/>
@@ -5166,12 +5250,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B43" s="56"/>
-      <c r="C43" s="80"/>
-      <c r="D43" s="83"/>
-      <c r="E43" s="63"/>
-      <c r="F43" s="63"/>
+    <row r="43" spans="2:58" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B43" s="47"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
       <c r="G43" s="15" t="s">
         <v>20</v>
       </c>
@@ -5231,18 +5315,18 @@
       <c r="BF43" s="18"/>
     </row>
     <row r="44" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B44" s="56" t="s">
-        <v>17</v>
-      </c>
-      <c r="C44" s="80"/>
-      <c r="D44" s="83">
+      <c r="B44" s="47" t="s">
+        <v>34</v>
+      </c>
+      <c r="C44" s="57"/>
+      <c r="D44" s="48">
         <f>SUM(AJ44:AK44)</f>
         <v>0</v>
       </c>
-      <c r="E44" s="63">
+      <c r="E44" s="49">
         <v>46097</v>
       </c>
-      <c r="F44" s="63">
+      <c r="F44" s="49">
         <v>46134</v>
       </c>
       <c r="G44" s="15" t="s">
@@ -5250,7 +5334,7 @@
       </c>
       <c r="H44" s="15">
         <f t="shared" si="0"/>
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="I44" s="25"/>
       <c r="J44" s="26"/>
@@ -5293,23 +5377,27 @@
       <c r="AM44" s="26"/>
       <c r="AN44" s="26"/>
       <c r="AO44" s="26"/>
-      <c r="AP44" s="26">
-        <v>63</v>
-      </c>
-      <c r="AQ44" s="26">
-        <v>63</v>
-      </c>
+      <c r="AP44" s="26"/>
+      <c r="AQ44" s="26"/>
       <c r="AR44" s="26"/>
       <c r="AS44" s="26"/>
-      <c r="AT44" s="26"/>
-      <c r="AU44" s="26"/>
+      <c r="AT44" s="26">
+        <v>24</v>
+      </c>
+      <c r="AU44" s="26">
+        <f>(63-AT44)/2</f>
+        <v>19.5</v>
+      </c>
       <c r="AV44" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="AW44" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="AX44" s="41"/>
+      <c r="AW44" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="AX44" s="26">
+        <f>63-AT44-AU44</f>
+        <v>19.5</v>
+      </c>
       <c r="AY44" s="41"/>
       <c r="AZ44" s="26"/>
       <c r="BA44" s="26"/>
@@ -5322,11 +5410,11 @@
       </c>
     </row>
     <row r="45" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B45" s="56"/>
-      <c r="C45" s="80"/>
-      <c r="D45" s="83"/>
-      <c r="E45" s="63"/>
-      <c r="F45" s="63"/>
+      <c r="B45" s="47"/>
+      <c r="C45" s="57"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="49"/>
+      <c r="F45" s="49"/>
       <c r="G45" s="15" t="s">
         <v>20</v>
       </c>
@@ -5386,18 +5474,18 @@
       <c r="BF45" s="18"/>
     </row>
     <row r="46" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B46" s="56" t="s">
-        <v>22</v>
-      </c>
-      <c r="C46" s="80"/>
-      <c r="D46" s="83">
+      <c r="B46" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="57"/>
+      <c r="D46" s="48">
         <f>SUM(AJ46:AL46)</f>
         <v>0</v>
       </c>
-      <c r="E46" s="63">
+      <c r="E46" s="49">
         <v>46097</v>
       </c>
-      <c r="F46" s="63">
+      <c r="F46" s="49">
         <v>46134</v>
       </c>
       <c r="G46" s="15" t="s">
@@ -5405,7 +5493,7 @@
       </c>
       <c r="H46" s="15">
         <f t="shared" si="0"/>
-        <v>75.599999999999994</v>
+        <v>0</v>
       </c>
       <c r="I46" s="25"/>
       <c r="J46" s="26"/>
@@ -5452,15 +5540,9 @@
       <c r="AM46" s="26"/>
       <c r="AN46" s="26"/>
       <c r="AO46" s="26"/>
-      <c r="AP46" s="26">
-        <v>25.2</v>
-      </c>
-      <c r="AQ46" s="26">
-        <v>25.2</v>
-      </c>
-      <c r="AR46" s="26">
-        <v>25.2</v>
-      </c>
+      <c r="AP46" s="26"/>
+      <c r="AQ46" s="26"/>
+      <c r="AR46" s="26"/>
       <c r="AS46" s="26"/>
       <c r="AT46" s="26"/>
       <c r="AU46" s="26"/>
@@ -5483,11 +5565,11 @@
       </c>
     </row>
     <row r="47" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B47" s="56"/>
-      <c r="C47" s="80"/>
-      <c r="D47" s="83"/>
-      <c r="E47" s="63"/>
-      <c r="F47" s="63"/>
+      <c r="B47" s="47"/>
+      <c r="C47" s="57"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="49"/>
+      <c r="F47" s="49"/>
       <c r="G47" s="15" t="s">
         <v>20</v>
       </c>
@@ -5547,18 +5629,18 @@
       <c r="BF47" s="18"/>
     </row>
     <row r="48" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B48" s="56" t="s">
+      <c r="B48" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="C48" s="80"/>
-      <c r="D48" s="83">
+      <c r="C48" s="57"/>
+      <c r="D48" s="48">
         <f>SUM(AK48:AL48,AM48)</f>
         <v>0</v>
       </c>
-      <c r="E48" s="63">
+      <c r="E48" s="49">
         <v>46097</v>
       </c>
-      <c r="F48" s="63">
+      <c r="F48" s="49">
         <v>46134</v>
       </c>
       <c r="G48" s="15" t="s">
@@ -5566,7 +5648,7 @@
       </c>
       <c r="H48" s="15">
         <f t="shared" si="0"/>
-        <v>11.399999999999999</v>
+        <v>0</v>
       </c>
       <c r="I48" s="25"/>
       <c r="J48" s="26"/>
@@ -5612,15 +5694,9 @@
       <c r="AN48" s="26"/>
       <c r="AO48" s="26"/>
       <c r="AP48" s="26"/>
-      <c r="AQ48" s="26">
-        <v>3.8</v>
-      </c>
-      <c r="AR48" s="26">
-        <v>3.8</v>
-      </c>
-      <c r="AS48" s="26">
-        <v>3.8</v>
-      </c>
+      <c r="AQ48" s="26"/>
+      <c r="AR48" s="26"/>
+      <c r="AS48" s="26"/>
       <c r="AT48" s="26"/>
       <c r="AU48" s="26"/>
       <c r="AV48" s="26" t="s">
@@ -5642,11 +5718,11 @@
       </c>
     </row>
     <row r="49" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B49" s="56"/>
-      <c r="C49" s="80"/>
-      <c r="D49" s="83"/>
-      <c r="E49" s="63"/>
-      <c r="F49" s="63"/>
+      <c r="B49" s="47"/>
+      <c r="C49" s="57"/>
+      <c r="D49" s="48"/>
+      <c r="E49" s="49"/>
+      <c r="F49" s="49"/>
       <c r="G49" s="15" t="s">
         <v>20</v>
       </c>
@@ -5706,18 +5782,18 @@
       <c r="BF49" s="18"/>
     </row>
     <row r="50" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B50" s="84" t="s">
+      <c r="B50" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="C50" s="80"/>
-      <c r="D50" s="85">
+      <c r="C50" s="57"/>
+      <c r="D50" s="62">
         <f>SUM(AL50:AO50)</f>
         <v>0</v>
       </c>
-      <c r="E50" s="63">
+      <c r="E50" s="49">
         <v>46097</v>
       </c>
-      <c r="F50" s="63">
+      <c r="F50" s="49">
         <v>46134</v>
       </c>
       <c r="G50" s="15" t="s">
@@ -5774,17 +5850,13 @@
       </c>
       <c r="AP50" s="26"/>
       <c r="AQ50" s="26"/>
-      <c r="AR50" s="26">
-        <v>15.75</v>
-      </c>
-      <c r="AS50" s="26">
-        <v>15.75</v>
-      </c>
+      <c r="AR50" s="26"/>
+      <c r="AS50" s="26"/>
       <c r="AT50" s="26">
-        <v>15.75</v>
+        <v>30</v>
       </c>
       <c r="AU50" s="26">
-        <v>15.75</v>
+        <v>33</v>
       </c>
       <c r="AV50" s="26" t="s">
         <v>19</v>
@@ -5805,11 +5877,11 @@
       </c>
     </row>
     <row r="51" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B51" s="84"/>
-      <c r="C51" s="80"/>
-      <c r="D51" s="85"/>
-      <c r="E51" s="63"/>
-      <c r="F51" s="63"/>
+      <c r="B51" s="61"/>
+      <c r="C51" s="57"/>
+      <c r="D51" s="62"/>
+      <c r="E51" s="49"/>
+      <c r="F51" s="49"/>
       <c r="G51" s="15" t="s">
         <v>20</v>
       </c>
@@ -5869,18 +5941,18 @@
       <c r="BF51" s="18"/>
     </row>
     <row r="52" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B52" s="56" t="s">
+      <c r="B52" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="C52" s="80"/>
-      <c r="D52" s="83">
+      <c r="C52" s="57"/>
+      <c r="D52" s="48">
         <f>SUM(AO52)</f>
         <v>0</v>
       </c>
-      <c r="E52" s="63">
+      <c r="E52" s="49">
         <v>46097</v>
       </c>
-      <c r="F52" s="63">
+      <c r="F52" s="49">
         <v>46134</v>
       </c>
       <c r="G52" s="15" t="s">
@@ -5956,11 +6028,11 @@
       </c>
     </row>
     <row r="53" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B53" s="56"/>
-      <c r="C53" s="80"/>
-      <c r="D53" s="83"/>
-      <c r="E53" s="63"/>
-      <c r="F53" s="63"/>
+      <c r="B53" s="47"/>
+      <c r="C53" s="57"/>
+      <c r="D53" s="48"/>
+      <c r="E53" s="49"/>
+      <c r="F53" s="49"/>
       <c r="G53" s="15" t="s">
         <v>20</v>
       </c>
@@ -6020,18 +6092,18 @@
       <c r="BF53" s="18"/>
     </row>
     <row r="54" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B54" s="56" t="s">
-        <v>26</v>
-      </c>
-      <c r="C54" s="80"/>
-      <c r="D54" s="83">
+      <c r="B54" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="C54" s="57"/>
+      <c r="D54" s="48">
         <f>SUM(AM54:AP54)</f>
-        <v>18.399999999999999</v>
-      </c>
-      <c r="E54" s="63">
+        <v>0</v>
+      </c>
+      <c r="E54" s="49">
         <v>46097</v>
       </c>
-      <c r="F54" s="63">
+      <c r="F54" s="49">
         <v>46134</v>
       </c>
       <c r="G54" s="15" t="s">
@@ -6039,7 +6111,7 @@
       </c>
       <c r="H54" s="15">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="I54" s="25"/>
       <c r="J54" s="26"/>
@@ -6085,24 +6157,32 @@
         <v>0</v>
       </c>
       <c r="AP54" s="26">
-        <v>18.399999999999999</v>
+        <v>0</v>
       </c>
       <c r="AQ54" s="26">
-        <v>18.399999999999999</v>
+        <v>0</v>
       </c>
       <c r="AR54" s="26">
-        <v>18.2</v>
+        <v>0</v>
       </c>
       <c r="AS54" s="26"/>
-      <c r="AT54" s="26"/>
-      <c r="AU54" s="26"/>
+      <c r="AT54" s="26">
+        <v>18</v>
+      </c>
+      <c r="AU54" s="26">
+        <f>(63-AT54)/2</f>
+        <v>22.5</v>
+      </c>
       <c r="AV54" s="26" t="s">
         <v>19</v>
       </c>
       <c r="AW54" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="AX54" s="26"/>
+      <c r="AX54" s="26">
+        <f>63-AT54-AU54</f>
+        <v>22.5</v>
+      </c>
       <c r="AY54" s="26"/>
       <c r="AZ54" s="26"/>
       <c r="BA54" s="26"/>
@@ -6115,11 +6195,11 @@
       </c>
     </row>
     <row r="55" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B55" s="56"/>
-      <c r="C55" s="80"/>
-      <c r="D55" s="83"/>
-      <c r="E55" s="63"/>
-      <c r="F55" s="63"/>
+      <c r="B55" s="47"/>
+      <c r="C55" s="57"/>
+      <c r="D55" s="48"/>
+      <c r="E55" s="49"/>
+      <c r="F55" s="49"/>
       <c r="G55" s="15" t="s">
         <v>20</v>
       </c>
@@ -6179,18 +6259,18 @@
       <c r="BF55" s="18"/>
     </row>
     <row r="56" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B56" s="56" t="s">
+      <c r="B56" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C56" s="80"/>
-      <c r="D56" s="83">
+      <c r="C56" s="57"/>
+      <c r="D56" s="48">
         <f>SUM(AO56:AQ56)</f>
         <v>0</v>
       </c>
-      <c r="E56" s="63">
+      <c r="E56" s="49">
         <v>46097</v>
       </c>
-      <c r="F56" s="63">
+      <c r="F56" s="49">
         <v>46134</v>
       </c>
       <c r="G56" s="15" t="s">
@@ -6198,7 +6278,7 @@
       </c>
       <c r="H56" s="15">
         <f t="shared" si="0"/>
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="I56" s="25"/>
       <c r="J56" s="26"/>
@@ -6236,25 +6316,13 @@
       <c r="AL56" s="26"/>
       <c r="AM56" s="26"/>
       <c r="AN56" s="26"/>
-      <c r="AO56" s="45">
-        <v>0</v>
-      </c>
-      <c r="AP56" s="45">
-        <v>0</v>
-      </c>
-      <c r="AQ56" s="45">
-        <v>0</v>
-      </c>
+      <c r="AO56" s="45"/>
+      <c r="AP56" s="45"/>
+      <c r="AQ56" s="45"/>
       <c r="AR56" s="26"/>
-      <c r="AS56" s="26">
-        <v>42</v>
-      </c>
-      <c r="AT56" s="26">
-        <v>42</v>
-      </c>
-      <c r="AU56" s="26">
-        <v>42</v>
-      </c>
+      <c r="AS56" s="26"/>
+      <c r="AT56" s="26"/>
+      <c r="AU56" s="26"/>
       <c r="AV56" s="26" t="s">
         <v>19</v>
       </c>
@@ -6274,11 +6342,11 @@
       </c>
     </row>
     <row r="57" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B57" s="56"/>
-      <c r="C57" s="80"/>
-      <c r="D57" s="83"/>
-      <c r="E57" s="63"/>
-      <c r="F57" s="63"/>
+      <c r="B57" s="47"/>
+      <c r="C57" s="57"/>
+      <c r="D57" s="48"/>
+      <c r="E57" s="49"/>
+      <c r="F57" s="49"/>
       <c r="G57" s="15" t="s">
         <v>20</v>
       </c>
@@ -6338,18 +6406,18 @@
       <c r="BF57" s="18"/>
     </row>
     <row r="58" spans="2:58" x14ac:dyDescent="0.3">
-      <c r="B58" s="56" t="s">
-        <v>28</v>
-      </c>
-      <c r="C58" s="80"/>
-      <c r="D58" s="83">
+      <c r="B58" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="C58" s="57"/>
+      <c r="D58" s="48">
         <f>SUM(AU58)</f>
         <v>0</v>
       </c>
-      <c r="E58" s="63">
+      <c r="E58" s="49">
         <v>46097</v>
       </c>
-      <c r="F58" s="63">
+      <c r="F58" s="49">
         <v>46134</v>
       </c>
       <c r="G58" s="15" t="s">
@@ -6357,7 +6425,7 @@
       </c>
       <c r="H58" s="15">
         <f t="shared" si="0"/>
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="I58" s="25"/>
       <c r="J58" s="26"/>
@@ -6411,10 +6479,10 @@
         <v>19</v>
       </c>
       <c r="AX58" s="26"/>
-      <c r="AY58" s="26"/>
-      <c r="AZ58" s="26">
-        <v>126</v>
-      </c>
+      <c r="AY58" s="26">
+        <v>63</v>
+      </c>
+      <c r="AZ58" s="26"/>
       <c r="BA58" s="26"/>
       <c r="BB58" s="26"/>
       <c r="BC58" s="26"/>
@@ -6425,11 +6493,11 @@
       </c>
     </row>
     <row r="59" spans="2:58" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="67"/>
-      <c r="C59" s="81"/>
-      <c r="D59" s="86"/>
-      <c r="E59" s="69"/>
-      <c r="F59" s="69"/>
+      <c r="B59" s="50"/>
+      <c r="C59" s="58"/>
+      <c r="D59" s="51"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
       <c r="G59" s="31" t="s">
         <v>20</v>
       </c>
@@ -6488,25 +6556,103 @@
       <c r="BE59" s="32"/>
       <c r="BF59" s="34"/>
     </row>
+    <row r="61" spans="2:58" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AM61" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="131">
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="F56:F57"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="E58:E59"/>
-    <mergeCell ref="F58:F59"/>
-    <mergeCell ref="F50:F51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="E54:E55"/>
-    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="I2:M2"/>
+    <mergeCell ref="N2:R2"/>
+    <mergeCell ref="S2:X2"/>
+    <mergeCell ref="Y2:AD2"/>
+    <mergeCell ref="AE2:AI2"/>
+    <mergeCell ref="AJ2:AO2"/>
+    <mergeCell ref="AP2:AU2"/>
+    <mergeCell ref="AV2:BA2"/>
+    <mergeCell ref="BB2:BF2"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C21"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C41"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="F38:F39"/>
     <mergeCell ref="B40:B41"/>
     <mergeCell ref="D40:D41"/>
     <mergeCell ref="E40:E41"/>
@@ -6531,96 +6677,23 @@
     <mergeCell ref="B50:B51"/>
     <mergeCell ref="D50:D51"/>
     <mergeCell ref="E50:E51"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="F34:F35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="F38:F39"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C41"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C21"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="I2:M2"/>
-    <mergeCell ref="N2:R2"/>
-    <mergeCell ref="S2:X2"/>
-    <mergeCell ref="Y2:AD2"/>
-    <mergeCell ref="AE2:AI2"/>
-    <mergeCell ref="AJ2:AO2"/>
-    <mergeCell ref="AP2:AU2"/>
-    <mergeCell ref="AV2:BA2"/>
-    <mergeCell ref="BB2:BF2"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="F56:F57"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="E58:E59"/>
+    <mergeCell ref="F58:F59"/>
+    <mergeCell ref="F50:F51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="E54:E55"/>
+    <mergeCell ref="F54:F55"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
style: formatar relatório do whatsapp e adicionar espaçamento
</commit_message>
<xml_diff>
--- a/Planejamento Previsto Geral.xlsx
+++ b/Planejamento Previsto Geral.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{273B33F0-FB2B-49BA-9978-078728594A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A28161-0591-4E75-A761-42F55829E805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="6" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="7" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="43">
   <si>
     <t>ATIVIDADE</t>
   </si>
@@ -128,6 +129,194 @@
   <si>
     <t>Reposição de pavimento asfáltico (m)</t>
   </si>
+  <si>
+    <r>
+      <t>Rem. Pavimento Asfáltico</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>816,0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 408 m²</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Implantação de PV</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>1,0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 3 und</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Escavação</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>335,9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 260 m³</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Reaterro Compactado</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>135,7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 256 m³</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Assentamento de Tubulação</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>233,0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 238 m</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Desmonte de Rocha</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>25,1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 20 m³</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Reposição Pav. Asfáltico</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>0,0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 238 m</t>
+    </r>
+  </si>
+  <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <r>
+      <t>251,7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <color rgb="FF6B7280"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t> / 372</t>
+    </r>
+  </si>
+  <si>
+    <t>=</t>
+  </si>
 </sst>
 </file>
 
@@ -138,7 +327,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,6 +362,39 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="6"/>
+      <color rgb="FF6B7280"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color rgb="FF6B7280"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF8B1A1A"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF6B7280"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF6B7280"/>
+      <name val="Georgia"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -545,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -771,6 +993,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5545,5 +5771,136 @@
     <mergeCell ref="F44:F45"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A3BBC00-76FA-47B4-B9B3-89C423AF1102}">
+  <dimension ref="G12:K34"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="42.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="12" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G12" s="77"/>
+    </row>
+    <row r="13" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G13" s="77"/>
+    </row>
+    <row r="14" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G14" s="77"/>
+    </row>
+    <row r="15" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G15" s="77"/>
+    </row>
+    <row r="16" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G16" s="77"/>
+    </row>
+    <row r="17" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G17" s="77"/>
+    </row>
+    <row r="18" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G18" s="77"/>
+    </row>
+    <row r="22" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G23" s="77" t="s">
+        <v>33</v>
+      </c>
+      <c r="H23">
+        <v>816</v>
+      </c>
+      <c r="I23">
+        <v>408</v>
+      </c>
+      <c r="J23">
+        <f>I23-H23</f>
+        <v>-408</v>
+      </c>
+    </row>
+    <row r="24" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G24" s="77" t="s">
+        <v>34</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G25" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25">
+        <v>335.9</v>
+      </c>
+      <c r="I25">
+        <v>260</v>
+      </c>
+      <c r="J25">
+        <f t="shared" ref="J24:K31" si="0">I25-H25</f>
+        <v>-75.899999999999977</v>
+      </c>
+    </row>
+    <row r="26" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G26" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26">
+        <v>135.69999999999999</v>
+      </c>
+      <c r="I26">
+        <v>256</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="0"/>
+        <v>120.30000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G27" s="77" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G28" s="77" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G29" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="H31" s="78" t="s">
+        <v>41</v>
+      </c>
+      <c r="I31">
+        <v>251.7</v>
+      </c>
+      <c r="J31">
+        <v>372</v>
+      </c>
+      <c r="K31">
+        <f t="shared" si="0"/>
+        <v>120.30000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>